<commit_message>
Updated figures for extreme binary system
</commit_message>
<xml_diff>
--- a/Raw_data/Conductivity for Extreme Binary Salt Mixtures.xlsx
+++ b/Raw_data/Conductivity for Extreme Binary Salt Mixtures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/877d0e272dd2d022/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1281409-DC85-49DC-BB5A-591CDCB1173F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D0A0B37F-A516-46BE-8F56-92DEDFF2E210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{F02FE19A-AB85-41E0-9205-59F6983E8A3F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="16">
   <si>
     <t>CaCl2 Conc (mM)</t>
   </si>
@@ -116,7 +116,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -132,6 +132,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -168,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -192,16 +198,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2179E617-F013-457D-9052-B2C83185DA78}">
-  <dimension ref="B2:L24"/>
+  <dimension ref="B2:L38"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
@@ -545,7 +549,7 @@
     <col min="4" max="4" width="25.53125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.1328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.46484375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.53125" bestFit="1" customWidth="1"/>
@@ -569,7 +573,7 @@
       <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="11"/>
+      <c r="G2" s="8"/>
       <c r="H2" s="2" t="s">
         <v>1</v>
       </c>
@@ -600,7 +604,7 @@
       <c r="E3">
         <v>2048.1999999999998</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3">
         <v>20.68</v>
       </c>
       <c r="H3" s="4">
@@ -610,10 +614,10 @@
         <f>H3*30</f>
         <v>30</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3">
         <v>8735.9</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3">
         <v>7906.3</v>
       </c>
       <c r="L3">
@@ -634,7 +638,7 @@
       <c r="E4">
         <v>3917</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4">
         <v>20.79</v>
       </c>
       <c r="H4" s="4">
@@ -644,10 +648,10 @@
         <f t="shared" ref="I4:I7" si="1">H4*30</f>
         <v>60</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4">
         <v>16261</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4">
         <v>14806</v>
       </c>
       <c r="L4">
@@ -668,7 +672,7 @@
       <c r="E5">
         <v>5776.7</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5">
         <v>20.92</v>
       </c>
       <c r="H5" s="4">
@@ -678,10 +682,10 @@
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5">
         <v>23478</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5">
         <v>21535</v>
       </c>
       <c r="L5">
@@ -702,7 +706,7 @@
       <c r="E6">
         <v>7518.5</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6">
         <v>21.03</v>
       </c>
       <c r="H6" s="4">
@@ -712,10 +716,10 @@
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6">
         <v>30232</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6">
         <v>27926</v>
       </c>
       <c r="L6">
@@ -757,21 +761,21 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="8" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B12" s="6" t="s">
@@ -787,7 +791,7 @@
         <v>15</v>
       </c>
       <c r="F12" s="6"/>
-      <c r="G12" s="12"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="6" t="s">
         <v>6</v>
       </c>
@@ -818,7 +822,7 @@
       <c r="F13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="13"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="7" t="s">
         <v>7</v>
       </c>
@@ -854,7 +858,7 @@
         <f>10-E14-D14</f>
         <v>9.4499999999999993</v>
       </c>
-      <c r="G14" s="13"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="7">
         <v>1</v>
       </c>
@@ -893,7 +897,7 @@
         <f>10-E15-D15</f>
         <v>8.9</v>
       </c>
-      <c r="G15" s="13"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="4">
         <v>2</v>
       </c>
@@ -932,7 +936,7 @@
         <f>10-E16-D16</f>
         <v>8.35</v>
       </c>
-      <c r="G16" s="13"/>
+      <c r="G16" s="7"/>
       <c r="H16" s="4">
         <v>3</v>
       </c>
@@ -971,7 +975,7 @@
         <f>10-E17-D17</f>
         <v>7.8</v>
       </c>
-      <c r="G17" s="13"/>
+      <c r="G17" s="7"/>
       <c r="H17" s="4">
         <v>4</v>
       </c>
@@ -1010,7 +1014,7 @@
         <f>10-E18-D18</f>
         <v>7.25</v>
       </c>
-      <c r="G18" s="13"/>
+      <c r="G18" s="7"/>
       <c r="H18" s="4">
         <v>5</v>
       </c>
@@ -1036,18 +1040,22 @@
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="7"/>
-      <c r="G19" s="13"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="4"/>
       <c r="K19" s="6"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="4"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B21" s="4"/>
@@ -1055,40 +1063,498 @@
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="7"/>
-      <c r="G21" s="13"/>
+      <c r="G21" s="7"/>
       <c r="H21" s="4"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="4"/>
+      <c r="B22" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G22" s="8"/>
+      <c r="H22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="4"/>
+      <c r="B23" s="4">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4">
+        <f>B23*30</f>
+        <v>30</v>
+      </c>
+      <c r="D23">
+        <v>6156.9</v>
+      </c>
+      <c r="E23">
+        <v>5642.6</v>
+      </c>
+      <c r="F23">
+        <v>21.19</v>
+      </c>
+      <c r="H23" s="4">
+        <v>1</v>
+      </c>
+      <c r="I23" s="4">
+        <f>H23*10</f>
+        <v>10</v>
+      </c>
+      <c r="J23">
+        <v>3313.3</v>
+      </c>
+      <c r="K23">
+        <v>3052.1</v>
+      </c>
+      <c r="L23">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="4"/>
+      <c r="B24" s="4">
+        <v>2</v>
+      </c>
+      <c r="C24" s="4">
+        <f t="shared" ref="C24:C27" si="6">B24*30</f>
+        <v>60</v>
+      </c>
+      <c r="D24">
+        <v>11524</v>
+      </c>
+      <c r="E24">
+        <v>10572</v>
+      </c>
+      <c r="F24">
+        <v>21.24</v>
+      </c>
+      <c r="H24" s="4">
+        <v>2</v>
+      </c>
+      <c r="I24" s="4">
+        <f t="shared" ref="I24:I27" si="7">H24*10</f>
+        <v>20</v>
+      </c>
+      <c r="J24">
+        <v>6037.3</v>
+      </c>
+      <c r="K24">
+        <v>5579.3</v>
+      </c>
+      <c r="L24">
+        <v>21.49</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B25" s="4">
+        <v>3</v>
+      </c>
+      <c r="C25" s="4">
+        <f t="shared" si="6"/>
+        <v>90</v>
+      </c>
+      <c r="D25">
+        <v>16656</v>
+      </c>
+      <c r="E25">
+        <v>15313</v>
+      </c>
+      <c r="F25">
+        <v>21.32</v>
+      </c>
+      <c r="H25" s="4">
+        <v>3</v>
+      </c>
+      <c r="I25" s="4">
+        <f t="shared" si="7"/>
+        <v>30</v>
+      </c>
+      <c r="J25">
+        <v>8687.7999999999993</v>
+      </c>
+      <c r="K25">
+        <v>8033.1</v>
+      </c>
+      <c r="L25">
+        <v>21.56</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B26" s="4">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4">
+        <f t="shared" si="6"/>
+        <v>120</v>
+      </c>
+      <c r="D26">
+        <v>21762</v>
+      </c>
+      <c r="E26">
+        <v>20036</v>
+      </c>
+      <c r="F26">
+        <v>21.38</v>
+      </c>
+      <c r="H26" s="4">
+        <v>4</v>
+      </c>
+      <c r="I26" s="4">
+        <f t="shared" si="7"/>
+        <v>40</v>
+      </c>
+      <c r="J26">
+        <v>11513</v>
+      </c>
+      <c r="K26">
+        <v>10659</v>
+      </c>
+      <c r="L26">
+        <v>21.65</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B27" s="5">
+        <v>5</v>
+      </c>
+      <c r="C27" s="5">
+        <f t="shared" si="6"/>
+        <v>150</v>
+      </c>
+      <c r="D27" s="1">
+        <v>26617</v>
+      </c>
+      <c r="E27" s="1">
+        <v>24585</v>
+      </c>
+      <c r="F27" s="1">
+        <v>21.54</v>
+      </c>
+      <c r="H27" s="5">
+        <v>5</v>
+      </c>
+      <c r="I27" s="5">
+        <f t="shared" si="7"/>
+        <v>50</v>
+      </c>
+      <c r="J27" s="1">
+        <v>13832</v>
+      </c>
+      <c r="K27" s="1">
+        <v>12865</v>
+      </c>
+      <c r="L27" s="1">
+        <v>21.78</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B30" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B32" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L32" s="6"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B33" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B34" s="7">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4">
+        <f>B34*30</f>
+        <v>30</v>
+      </c>
+      <c r="D34" s="6">
+        <f>B34*10/200</f>
+        <v>0.05</v>
+      </c>
+      <c r="E34" s="6">
+        <f>C34*10/200</f>
+        <v>1.5</v>
+      </c>
+      <c r="F34" s="7">
+        <f>10-E34-D34</f>
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7">
+        <v>1</v>
+      </c>
+      <c r="I34" s="7">
+        <v>10</v>
+      </c>
+      <c r="J34" s="6">
+        <f>H34*10/200</f>
+        <v>0.05</v>
+      </c>
+      <c r="K34" s="6">
+        <f>I34*10/200</f>
+        <v>0.5</v>
+      </c>
+      <c r="L34" s="7">
+        <f>10-K34-J34</f>
+        <v>9.4499999999999993</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B35" s="4">
+        <v>2</v>
+      </c>
+      <c r="C35" s="4">
+        <f t="shared" ref="C35:C38" si="8">B35*30</f>
+        <v>60</v>
+      </c>
+      <c r="D35" s="6">
+        <f t="shared" ref="D35:D38" si="9">B35*10/200</f>
+        <v>0.1</v>
+      </c>
+      <c r="E35" s="6">
+        <f t="shared" ref="E35:E38" si="10">C35*10/200</f>
+        <v>3</v>
+      </c>
+      <c r="F35" s="7">
+        <f>10-E35-D35</f>
+        <v>6.9</v>
+      </c>
+      <c r="G35" s="7"/>
+      <c r="H35" s="4">
+        <v>2</v>
+      </c>
+      <c r="I35" s="4">
+        <v>20</v>
+      </c>
+      <c r="J35" s="6">
+        <f t="shared" ref="J35:J38" si="11">H35*10/200</f>
+        <v>0.1</v>
+      </c>
+      <c r="K35" s="6">
+        <f t="shared" ref="K35:K38" si="12">I35*10/200</f>
+        <v>1</v>
+      </c>
+      <c r="L35" s="7">
+        <f>10-K35-J35</f>
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B36" s="4">
+        <v>3</v>
+      </c>
+      <c r="C36" s="4">
+        <f t="shared" si="8"/>
+        <v>90</v>
+      </c>
+      <c r="D36" s="6">
+        <f t="shared" si="9"/>
+        <v>0.15</v>
+      </c>
+      <c r="E36" s="6">
+        <f t="shared" si="10"/>
+        <v>4.5</v>
+      </c>
+      <c r="F36" s="7">
+        <f>10-E36-D36</f>
+        <v>5.35</v>
+      </c>
+      <c r="G36" s="7"/>
+      <c r="H36" s="4">
+        <v>3</v>
+      </c>
+      <c r="I36" s="4">
+        <v>30</v>
+      </c>
+      <c r="J36" s="6">
+        <f t="shared" si="11"/>
+        <v>0.15</v>
+      </c>
+      <c r="K36" s="6">
+        <f t="shared" si="12"/>
+        <v>1.5</v>
+      </c>
+      <c r="L36" s="7">
+        <f>10-K36-J36</f>
+        <v>8.35</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B37" s="4">
+        <v>4</v>
+      </c>
+      <c r="C37" s="4">
+        <f t="shared" si="8"/>
+        <v>120</v>
+      </c>
+      <c r="D37" s="6">
+        <f t="shared" si="9"/>
+        <v>0.2</v>
+      </c>
+      <c r="E37" s="6">
+        <f t="shared" si="10"/>
+        <v>6</v>
+      </c>
+      <c r="F37" s="7">
+        <f>10-E37-D37</f>
+        <v>3.8</v>
+      </c>
+      <c r="G37" s="7"/>
+      <c r="H37" s="4">
+        <v>4</v>
+      </c>
+      <c r="I37" s="4">
+        <v>40</v>
+      </c>
+      <c r="J37" s="6">
+        <f t="shared" si="11"/>
+        <v>0.2</v>
+      </c>
+      <c r="K37" s="6">
+        <f t="shared" si="12"/>
+        <v>2</v>
+      </c>
+      <c r="L37" s="7">
+        <f>10-K37-J37</f>
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B38" s="4">
+        <v>5</v>
+      </c>
+      <c r="C38" s="11">
+        <f t="shared" si="8"/>
+        <v>150</v>
+      </c>
+      <c r="D38" s="6">
+        <f t="shared" si="9"/>
+        <v>0.25</v>
+      </c>
+      <c r="E38" s="6">
+        <f t="shared" si="10"/>
+        <v>7.5</v>
+      </c>
+      <c r="F38" s="7">
+        <f>10-E38-D38</f>
+        <v>2.25</v>
+      </c>
+      <c r="G38" s="7"/>
+      <c r="H38" s="4">
+        <v>5</v>
+      </c>
+      <c r="I38" s="4">
+        <v>50</v>
+      </c>
+      <c r="J38" s="6">
+        <f t="shared" si="11"/>
+        <v>0.25</v>
+      </c>
+      <c r="K38" s="6">
+        <f t="shared" si="12"/>
+        <v>2.5</v>
+      </c>
+      <c r="L38" s="7">
+        <f>10-K38-J38</f>
+        <v>7.25</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="H10:L10"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="H30:L30"/>
+    <mergeCell ref="B20:L20"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>